<commit_message>
Complete Asset Accuracy tab: real reconciliation, replacement matching, review flags, interactive map
</commit_message>
<xml_diff>
--- a/data/coretex_equipment_records.xlsx
+++ b/data/coretex_equipment_records.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L153"/>
+  <dimension ref="A1:M153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -452,6 +452,7 @@
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -515,6 +516,11 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Status Change Date</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -577,6 +583,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>2015-07-17</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -639,6 +650,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>2017-02-17</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -701,6 +717,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>2019-08-25</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -763,6 +784,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>2018-07-29</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -822,7 +848,12 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Inactive</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
         </is>
       </c>
     </row>
@@ -887,6 +918,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>2015-01-08</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -949,6 +985,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>2018-02-28</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1011,6 +1052,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>2015-11-19</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1073,6 +1119,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>2019-04-26</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1135,6 +1186,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>2013-03-21</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1197,6 +1253,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>2014-06-12</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1256,7 +1317,12 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Inactive</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-18</t>
         </is>
       </c>
     </row>
@@ -1321,6 +1387,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>2018-09-24</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1383,6 +1454,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>2014-12-11</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1442,7 +1518,12 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>2024-09-17</t>
         </is>
       </c>
     </row>
@@ -1507,6 +1588,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>2021-02-03</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1569,6 +1655,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>2021-06-18</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1631,6 +1722,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>2015-04-24</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1690,7 +1786,12 @@
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>2017-08-26</t>
         </is>
       </c>
     </row>
@@ -1755,6 +1856,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>2015-11-02</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1817,6 +1923,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>2018-12-16</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1879,6 +1990,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>2015-12-10</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1941,6 +2057,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>2019-10-13</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2003,6 +2124,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>2021-06-06</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2065,6 +2191,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>2015-09-25</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2127,6 +2258,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>2018-03-02</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2189,6 +2325,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>2025-05-18</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2251,6 +2392,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>2022-01-05</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2313,6 +2459,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>2022-08-09</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2375,6 +2526,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>2024-02-27</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2437,6 +2593,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>2024-01-10</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2499,6 +2660,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>2011-12-23</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2561,6 +2727,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>2016-10-09</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2623,6 +2794,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>2013-12-09</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2685,6 +2861,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>2023-04-07</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2747,6 +2928,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>2015-05-23</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2809,6 +2995,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>2022-08-04</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2871,6 +3062,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>2020-08-16</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2930,7 +3126,12 @@
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Inactive</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-22</t>
         </is>
       </c>
     </row>
@@ -2995,6 +3196,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>2018-09-15</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3054,7 +3260,12 @@
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>2021-03-09</t>
         </is>
       </c>
     </row>
@@ -3119,6 +3330,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>2019-03-29</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3181,6 +3397,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>2019-02-11</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3243,6 +3464,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>2017-09-08</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3302,7 +3528,12 @@
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Inactive</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-11</t>
         </is>
       </c>
     </row>
@@ -3367,6 +3598,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M47" s="2" t="inlineStr">
+        <is>
+          <t>2021-12-31</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3429,6 +3665,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-12</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3491,6 +3732,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M49" s="2" t="inlineStr">
+        <is>
+          <t>2018-12-09</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3553,6 +3799,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>2014-05-10</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3615,6 +3866,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M51" s="2" t="inlineStr">
+        <is>
+          <t>2019-11-24</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3677,6 +3933,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>2010-07-28</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3739,6 +4000,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M53" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-09</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3798,7 +4064,12 @@
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>2021-05-19</t>
         </is>
       </c>
     </row>
@@ -3863,6 +4134,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M55" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3925,6 +4201,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>2020-09-21</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -3987,6 +4268,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M57" s="2" t="inlineStr">
+        <is>
+          <t>2016-04-10</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -4049,6 +4335,11 @@
           <t>Inactive</t>
         </is>
       </c>
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-14</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -4111,6 +4402,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M59" s="2" t="inlineStr">
+        <is>
+          <t>2020-02-26</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -4173,6 +4469,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M60" s="2" t="inlineStr">
+        <is>
+          <t>2023-08-08</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -4235,6 +4536,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M61" s="2" t="inlineStr">
+        <is>
+          <t>2022-01-14</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -4294,7 +4600,12 @@
       </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M62" s="2" t="inlineStr">
+        <is>
+          <t>2014-09-06</t>
         </is>
       </c>
     </row>
@@ -4359,6 +4670,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>2018-09-05</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -4421,6 +4737,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M64" s="2" t="inlineStr">
+        <is>
+          <t>2013-08-12</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -4483,6 +4804,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M65" s="2" t="inlineStr">
+        <is>
+          <t>2019-12-13</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -4545,6 +4871,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M66" s="2" t="inlineStr">
+        <is>
+          <t>2023-08-25</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -4607,6 +4938,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M67" s="2" t="inlineStr">
+        <is>
+          <t>2014-11-22</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -4666,7 +5002,12 @@
       </c>
       <c r="L68" s="2" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>2020-06-06</t>
         </is>
       </c>
     </row>
@@ -4731,6 +5072,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M69" s="2" t="inlineStr">
+        <is>
+          <t>2016-09-23</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -4793,6 +5139,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M70" s="2" t="inlineStr">
+        <is>
+          <t>2016-12-30</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -4855,6 +5206,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M71" s="2" t="inlineStr">
+        <is>
+          <t>2025-02-19</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -4917,6 +5273,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M72" s="2" t="inlineStr">
+        <is>
+          <t>2015-09-24</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -4979,6 +5340,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M73" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-18</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -5041,6 +5407,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M74" s="2" t="inlineStr">
+        <is>
+          <t>2024-01-10</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -5103,6 +5474,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M75" s="2" t="inlineStr">
+        <is>
+          <t>2022-04-02</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -5165,6 +5541,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M76" s="2" t="inlineStr">
+        <is>
+          <t>2007-04-25</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -5227,6 +5608,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M77" s="2" t="inlineStr">
+        <is>
+          <t>2016-08-13</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -5289,6 +5675,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>2015-10-17</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -5351,6 +5742,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M79" s="2" t="inlineStr">
+        <is>
+          <t>2015-05-01</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -5413,6 +5809,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M80" s="2" t="inlineStr">
+        <is>
+          <t>2014-05-06</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -5475,6 +5876,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M81" s="2" t="inlineStr">
+        <is>
+          <t>2019-09-08</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -5537,6 +5943,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M82" s="2" t="inlineStr">
+        <is>
+          <t>2017-02-27</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -5599,6 +6010,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M83" s="2" t="inlineStr">
+        <is>
+          <t>2023-09-04</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -5661,6 +6077,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M84" s="2" t="inlineStr">
+        <is>
+          <t>2017-06-04</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -5723,6 +6144,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M85" s="2" t="inlineStr">
+        <is>
+          <t>2021-03-21</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -5785,6 +6211,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M86" s="2" t="inlineStr">
+        <is>
+          <t>2023-12-10</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -5847,6 +6278,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M87" s="2" t="inlineStr">
+        <is>
+          <t>2013-04-02</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -5909,6 +6345,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M88" s="2" t="inlineStr">
+        <is>
+          <t>2016-12-30</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -5971,6 +6412,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M89" s="2" t="inlineStr">
+        <is>
+          <t>2018-10-16</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -6033,6 +6479,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M90" s="2" t="inlineStr">
+        <is>
+          <t>2015-12-20</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -6095,6 +6546,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M91" s="2" t="inlineStr">
+        <is>
+          <t>2022-01-17</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -6157,6 +6613,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M92" s="2" t="inlineStr">
+        <is>
+          <t>2019-03-11</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -6219,6 +6680,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M93" s="2" t="inlineStr">
+        <is>
+          <t>2016-10-10</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -6278,7 +6744,12 @@
       </c>
       <c r="L94" s="2" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M94" s="2" t="inlineStr">
+        <is>
+          <t>2022-12-10</t>
         </is>
       </c>
     </row>
@@ -6343,6 +6814,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M95" s="2" t="inlineStr">
+        <is>
+          <t>2011-03-28</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -6405,6 +6881,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M96" s="2" t="inlineStr">
+        <is>
+          <t>2013-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -6467,6 +6948,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M97" s="2" t="inlineStr">
+        <is>
+          <t>2017-06-27</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -6529,6 +7015,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M98" s="2" t="inlineStr">
+        <is>
+          <t>2023-06-03</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -6553,17 +7044,17 @@
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>WA088</t>
+          <t>WA100</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>3 Warehouse Ln</t>
+          <t>12 Settlers Ave</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>Morley</t>
+          <t>Baldivis</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr">
@@ -6573,7 +7064,7 @@
       </c>
       <c r="I99" s="2" t="inlineStr">
         <is>
-          <t>6340</t>
+          <t>6171</t>
         </is>
       </c>
       <c r="J99" s="2" t="inlineStr">
@@ -6589,6 +7080,11 @@
       <c r="L99" s="2" t="inlineStr">
         <is>
           <t>Active</t>
+        </is>
+      </c>
+      <c r="M99" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-29</t>
         </is>
       </c>
     </row>
@@ -6653,6 +7149,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M100" s="2" t="inlineStr">
+        <is>
+          <t>2020-06-24</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -6715,6 +7216,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M101" s="2" t="inlineStr">
+        <is>
+          <t>2015-07-19</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -6777,6 +7283,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M102" s="2" t="inlineStr">
+        <is>
+          <t>2021-07-08</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -6839,6 +7350,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M103" s="2" t="inlineStr">
+        <is>
+          <t>2025-05-20</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -6901,6 +7417,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M104" s="2" t="inlineStr">
+        <is>
+          <t>2014-04-03</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -6963,6 +7484,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M105" s="2" t="inlineStr">
+        <is>
+          <t>2020-08-11</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -7022,7 +7548,12 @@
       </c>
       <c r="L106" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Inactive</t>
+        </is>
+      </c>
+      <c r="M106" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-20</t>
         </is>
       </c>
     </row>
@@ -7087,6 +7618,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M107" s="2" t="inlineStr">
+        <is>
+          <t>2016-07-15</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -7149,6 +7685,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M108" s="2" t="inlineStr">
+        <is>
+          <t>2018-09-05</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -7211,6 +7752,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M109" s="2" t="inlineStr">
+        <is>
+          <t>2017-07-05</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -7273,6 +7819,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M110" s="2" t="inlineStr">
+        <is>
+          <t>2013-11-05</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -7335,6 +7886,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M111" s="2" t="inlineStr">
+        <is>
+          <t>2018-01-22</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -7397,6 +7953,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M112" s="2" t="inlineStr">
+        <is>
+          <t>2022-10-16</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -7459,6 +8020,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M113" s="2" t="inlineStr">
+        <is>
+          <t>2020-07-06</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -7518,7 +8084,12 @@
       </c>
       <c r="L114" s="2" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M114" s="2" t="inlineStr">
+        <is>
+          <t>2013-02-20</t>
         </is>
       </c>
     </row>
@@ -7583,6 +8154,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M115" s="2" t="inlineStr">
+        <is>
+          <t>2016-06-26</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -7645,6 +8221,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M116" s="2" t="inlineStr">
+        <is>
+          <t>2024-04-04</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -7707,6 +8288,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M117" s="2" t="inlineStr">
+        <is>
+          <t>2018-07-31</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -7769,6 +8355,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M118" s="2" t="inlineStr">
+        <is>
+          <t>2016-08-28</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -7831,6 +8422,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M119" s="2" t="inlineStr">
+        <is>
+          <t>2014-05-05</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -7893,6 +8489,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M120" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-19</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -7955,6 +8556,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M121" s="2" t="inlineStr">
+        <is>
+          <t>2013-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -8017,6 +8623,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M122" s="2" t="inlineStr">
+        <is>
+          <t>2024-01-07</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -8079,6 +8690,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M123" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-19</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -8141,6 +8757,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M124" s="2" t="inlineStr">
+        <is>
+          <t>2023-02-06</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -8203,6 +8824,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M125" s="2" t="inlineStr">
+        <is>
+          <t>2016-06-13</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -8265,6 +8891,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M126" s="2" t="inlineStr">
+        <is>
+          <t>2016-11-11</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -8327,6 +8958,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M127" s="2" t="inlineStr">
+        <is>
+          <t>2017-08-23</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -8389,6 +9025,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M128" s="2" t="inlineStr">
+        <is>
+          <t>2024-11-09</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -8451,6 +9092,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M129" s="2" t="inlineStr">
+        <is>
+          <t>2022-01-10</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -8513,6 +9159,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M130" s="2" t="inlineStr">
+        <is>
+          <t>2016-08-04</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -8575,6 +9226,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M131" s="2" t="inlineStr">
+        <is>
+          <t>2025-02-13</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -8637,6 +9293,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M132" s="2" t="inlineStr">
+        <is>
+          <t>2014-10-22</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -8699,6 +9360,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M133" s="2" t="inlineStr">
+        <is>
+          <t>2017-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -8761,6 +9427,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M134" s="2" t="inlineStr">
+        <is>
+          <t>2013-03-01</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -8823,6 +9494,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M135" s="2" t="inlineStr">
+        <is>
+          <t>2024-12-01</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -8882,7 +9558,12 @@
       </c>
       <c r="L136" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Inactive</t>
+        </is>
+      </c>
+      <c r="M136" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-20</t>
         </is>
       </c>
     </row>
@@ -8947,6 +9628,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M137" s="2" t="inlineStr">
+        <is>
+          <t>2018-01-22</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -9009,6 +9695,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M138" s="2" t="inlineStr">
+        <is>
+          <t>2018-02-06</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -9071,6 +9762,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M139" s="2" t="inlineStr">
+        <is>
+          <t>2006-08-31</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -9130,7 +9826,12 @@
       </c>
       <c r="L140" s="2" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M140" s="2" t="inlineStr">
+        <is>
+          <t>2019-06-08</t>
         </is>
       </c>
     </row>
@@ -9192,7 +9893,12 @@
       </c>
       <c r="L141" s="2" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M141" s="2" t="inlineStr">
+        <is>
+          <t>2014-07-30</t>
         </is>
       </c>
     </row>
@@ -9257,6 +9963,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M142" s="2" t="inlineStr">
+        <is>
+          <t>2017-07-01</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -9316,7 +10027,12 @@
       </c>
       <c r="L143" s="2" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M143" s="2" t="inlineStr">
+        <is>
+          <t>2023-03-07</t>
         </is>
       </c>
     </row>
@@ -9381,6 +10097,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M144" s="2" t="inlineStr">
+        <is>
+          <t>2016-06-09</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -9443,6 +10164,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M145" s="2" t="inlineStr">
+        <is>
+          <t>2016-09-15</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -9505,6 +10231,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M146" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-17</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -9567,6 +10298,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M147" s="2" t="inlineStr">
+        <is>
+          <t>2014-09-16</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -9629,6 +10365,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M148" s="2" t="inlineStr">
+        <is>
+          <t>2013-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -9691,6 +10432,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M149" s="2" t="inlineStr">
+        <is>
+          <t>2024-12-06</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -9753,6 +10499,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M150" s="2" t="inlineStr">
+        <is>
+          <t>2021-06-24</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -9815,6 +10566,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M151" s="2" t="inlineStr">
+        <is>
+          <t>2013-09-30</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -9877,6 +10633,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="M152" s="2" t="inlineStr">
+        <is>
+          <t>2019-05-18</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -9936,7 +10697,12 @@
       </c>
       <c r="L153" s="2" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M153" s="2" t="inlineStr">
+        <is>
+          <t>2022-11-17</t>
         </is>
       </c>
     </row>

</xml_diff>